<commit_message>
Added new RDF data schemes and visual schemes for employment-table01-05, fixed XLSX spreadsheets for employment-table01-03
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/employment-table01.xlsx
+++ b/sources/table_normalization/xlsx/employment-table01.xlsx
@@ -122,22 +122,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -450,19 +451,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="5"/>
+      <c r="K1" s="5"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
@@ -470,86 +471,99 @@
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="5"/>
-      <c r="K4" s="6" t="s">
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="7" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A5" s="5"/>
-      <c r="B5" s="7"/>
-      <c r="C5" s="5" t="s">
+      <c r="A5" s="6"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5" t="s">
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
     </row>
     <row r="6" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="5"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
+      <c r="A6" s="6"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6"/>
       <c r="E6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="H6" s="8" t="s">
+      <c r="H6" s="4" t="s">
         <v>11</v>
       </c>
       <c r="I6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="J6" s="8" t="s">
+      <c r="J6" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="K6" s="5"/>
+      <c r="K6" s="6"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
-      <c r="K8" s="1"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9">
@@ -3037,22 +3051,25 @@
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A81" s="2" t="s">
+      <c r="A81" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B81" s="2"/>
-      <c r="C81" s="2"/>
-      <c r="D81" s="2"/>
-      <c r="E81" s="2"/>
-      <c r="F81" s="2"/>
-      <c r="G81" s="2"/>
-      <c r="H81" s="2"/>
-      <c r="I81" s="2"/>
-      <c r="J81" s="2"/>
-      <c r="K81" s="2"/>
+      <c r="B81" s="5"/>
+      <c r="C81" s="5"/>
+      <c r="D81" s="5"/>
+      <c r="E81" s="5"/>
+      <c r="F81" s="5"/>
+      <c r="G81" s="5"/>
+      <c r="H81" s="5"/>
+      <c r="I81" s="5"/>
+      <c r="J81" s="5"/>
+      <c r="K81" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A81:K81"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="D5:D6"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="E5:H5"/>
     <mergeCell ref="C5:C6"/>
@@ -3060,9 +3077,6 @@
     <mergeCell ref="K4:K6"/>
     <mergeCell ref="A4:A6"/>
     <mergeCell ref="B4:B6"/>
-    <mergeCell ref="A81:K81"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="D5:D6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>